<commit_message>
Shorts phase 1 (work in progress): session chart, FRED chart, tests
Today's session on the move beat (item 4), read off Yahoo's five-minute
prices and never synthesised; the macro short's series off FRED's public
CSV with recessions shaded, and the print checked against it before
approval (item 6). The earnings quarter chart now draws from the figures
it prints. Tests updated for the new short layout. Not for merge until
the re-rendered frames are approved.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PtFQaojNjukBZRpdj68CaY
</commit_message>
<xml_diff>
--- a/templates/dennis_data_template.xlsx
+++ b/templates/dennis_data_template.xlsx
@@ -329,7 +329,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="13" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -438,6 +438,10 @@
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="7" fillId="16" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="7" fillId="15" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3405,7 +3409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17.28515625" bestFit="1" customWidth="1" style="90" min="1" max="1"/>
@@ -4759,6 +4763,45 @@
       <c r="J34" s="7" t="inlineStr">
         <is>
           <t>computed</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>fiscal_year</t>
+        </is>
+      </c>
+      <c r="B35" s="94" t="inlineStr">
+        <is>
+          <t>Fiscal year (labels the column)</t>
+        </is>
+      </c>
+      <c r="C35" s="95">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_FISCAL_Y", IQ_FY - 4)</f>
+        <v/>
+      </c>
+      <c r="D35" s="95">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_FISCAL_Y", IQ_FY - 3)</f>
+        <v/>
+      </c>
+      <c r="E35" s="95">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_FISCAL_Y", IQ_FY - 2)</f>
+        <v/>
+      </c>
+      <c r="F35" s="95">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_FISCAL_Y", IQ_FY - 1)</f>
+        <v/>
+      </c>
+      <c r="G35" s="95">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_FISCAL_Y", IQ_FY)</f>
+        <v/>
+      </c>
+      <c r="H35" s="95" t="n"/>
+      <c r="I35" s="96" t="n"/>
+      <c r="J35" s="7" t="inlineStr">
+        <is>
+          <t>TR.FiscalYear</t>
         </is>
       </c>
     </row>
@@ -4777,7 +4820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="90" min="1" max="1"/>
@@ -5602,35 +5645,35 @@
         </is>
       </c>
       <c r="C20">
-        <f>IF(C18="","",C18-C17)</f>
+        <f>IF(C19="","",C19-C18)</f>
         <v/>
       </c>
       <c r="D20">
-        <f>IF(D18="","",D18-D17)</f>
+        <f>IF(D19="","",D19-D18)</f>
         <v/>
       </c>
       <c r="E20">
-        <f>IF(E18="","",E18-E17)</f>
+        <f>IF(E19="","",E19-E18)</f>
         <v/>
       </c>
       <c r="F20">
-        <f>IF(F18="","",F18-F17)</f>
+        <f>IF(F19="","",F19-F18)</f>
         <v/>
       </c>
       <c r="G20">
-        <f>IF(G18="","",G18-G17)</f>
+        <f>IF(G19="","",G19-G18)</f>
         <v/>
       </c>
       <c r="H20">
-        <f>IF(H18="","",H18-H17)</f>
+        <f>IF(H19="","",H19-H18)</f>
         <v/>
       </c>
       <c r="I20">
-        <f>IF(I18="","",I18-I17)</f>
+        <f>IF(I19="","",I19-I18)</f>
         <v/>
       </c>
       <c r="J20">
-        <f>IF(J18="","",J18-J17)</f>
+        <f>IF(J19="","",J19-J18)</f>
         <v/>
       </c>
       <c r="K20" t="inlineStr">
@@ -5783,6 +5826,251 @@
       <c r="K23" t="inlineStr">
         <is>
           <t>computed</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="97" t="inlineStr">
+        <is>
+          <t>eps_street</t>
+        </is>
+      </c>
+      <c r="B24" s="97" t="inlineStr">
+        <is>
+          <t>EPS actual (street basis)</t>
+        </is>
+      </c>
+      <c r="C24" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_EPS_ACT", IQ_FQ - 7)</f>
+        <v/>
+      </c>
+      <c r="D24" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_EPS_ACT", IQ_FQ - 6)</f>
+        <v/>
+      </c>
+      <c r="E24" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_EPS_ACT", IQ_FQ - 5)</f>
+        <v/>
+      </c>
+      <c r="F24" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_EPS_ACT", IQ_FQ - 4)</f>
+        <v/>
+      </c>
+      <c r="G24" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_EPS_ACT", IQ_FQ - 3)</f>
+        <v/>
+      </c>
+      <c r="H24" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_EPS_ACT", IQ_FQ - 2)</f>
+        <v/>
+      </c>
+      <c r="I24" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_EPS_ACT", IQ_FQ - 1)</f>
+        <v/>
+      </c>
+      <c r="J24" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_EPS_ACT", IQ_FQ)</f>
+        <v/>
+      </c>
+      <c r="K24" s="97" t="inlineStr">
+        <is>
+          <t>TR.EPSActValue</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="97" t="inlineStr">
+        <is>
+          <t>eps_consensus</t>
+        </is>
+      </c>
+      <c r="B25" s="97" t="inlineStr">
+        <is>
+          <t>EPS estimate (consensus mean)</t>
+        </is>
+      </c>
+      <c r="C25" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_EPS_EST", IQ_FQ - 7)</f>
+        <v/>
+      </c>
+      <c r="D25" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_EPS_EST", IQ_FQ - 6)</f>
+        <v/>
+      </c>
+      <c r="E25" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_EPS_EST", IQ_FQ - 5)</f>
+        <v/>
+      </c>
+      <c r="F25" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_EPS_EST", IQ_FQ - 4)</f>
+        <v/>
+      </c>
+      <c r="G25" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_EPS_EST", IQ_FQ - 3)</f>
+        <v/>
+      </c>
+      <c r="H25" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_EPS_EST", IQ_FQ - 2)</f>
+        <v/>
+      </c>
+      <c r="I25" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_EPS_EST", IQ_FQ - 1)</f>
+        <v/>
+      </c>
+      <c r="J25" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_EPS_EST", IQ_FQ)</f>
+        <v/>
+      </c>
+      <c r="K25" s="97" t="inlineStr">
+        <is>
+          <t>TR.EPSMean</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="97" t="inlineStr">
+        <is>
+          <t>revenue_consensus</t>
+        </is>
+      </c>
+      <c r="B26" s="97" t="inlineStr">
+        <is>
+          <t>Revenue estimate (consensus mean)</t>
+        </is>
+      </c>
+      <c r="C26" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_REVENUE_EST", IQ_FQ - 7)</f>
+        <v/>
+      </c>
+      <c r="D26" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_REVENUE_EST", IQ_FQ - 6)</f>
+        <v/>
+      </c>
+      <c r="E26" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_REVENUE_EST", IQ_FQ - 5)</f>
+        <v/>
+      </c>
+      <c r="F26" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_REVENUE_EST", IQ_FQ - 4)</f>
+        <v/>
+      </c>
+      <c r="G26" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_REVENUE_EST", IQ_FQ - 3)</f>
+        <v/>
+      </c>
+      <c r="H26" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_REVENUE_EST", IQ_FQ - 2)</f>
+        <v/>
+      </c>
+      <c r="I26" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_REVENUE_EST", IQ_FQ - 1)</f>
+        <v/>
+      </c>
+      <c r="J26" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_REVENUE_EST", IQ_FQ)</f>
+        <v/>
+      </c>
+      <c r="K26" s="97" t="inlineStr">
+        <is>
+          <t>TR.RevenueMean</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="97" t="inlineStr">
+        <is>
+          <t>fiscal_year</t>
+        </is>
+      </c>
+      <c r="B27" s="97" t="inlineStr">
+        <is>
+          <t>Fiscal year (labels the column)</t>
+        </is>
+      </c>
+      <c r="C27" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_FISCAL_Y", IQ_FQ - 7)</f>
+        <v/>
+      </c>
+      <c r="D27" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_FISCAL_Y", IQ_FQ - 6)</f>
+        <v/>
+      </c>
+      <c r="E27" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_FISCAL_Y", IQ_FQ - 5)</f>
+        <v/>
+      </c>
+      <c r="F27" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_FISCAL_Y", IQ_FQ - 4)</f>
+        <v/>
+      </c>
+      <c r="G27" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_FISCAL_Y", IQ_FQ - 3)</f>
+        <v/>
+      </c>
+      <c r="H27" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_FISCAL_Y", IQ_FQ - 2)</f>
+        <v/>
+      </c>
+      <c r="I27" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_FISCAL_Y", IQ_FQ - 1)</f>
+        <v/>
+      </c>
+      <c r="J27" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_FISCAL_Y", IQ_FQ)</f>
+        <v/>
+      </c>
+      <c r="K27" s="97" t="inlineStr">
+        <is>
+          <t>TR.FiscalYear</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="97" t="inlineStr">
+        <is>
+          <t>fiscal_quarter</t>
+        </is>
+      </c>
+      <c r="B28" s="97" t="inlineStr">
+        <is>
+          <t>Fiscal quarter (labels the column)</t>
+        </is>
+      </c>
+      <c r="C28" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_FISCAL_Q", IQ_FQ - 7)</f>
+        <v/>
+      </c>
+      <c r="D28" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_FISCAL_Q", IQ_FQ - 6)</f>
+        <v/>
+      </c>
+      <c r="E28" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_FISCAL_Q", IQ_FQ - 5)</f>
+        <v/>
+      </c>
+      <c r="F28" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_FISCAL_Q", IQ_FQ - 4)</f>
+        <v/>
+      </c>
+      <c r="G28" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_FISCAL_Q", IQ_FQ - 3)</f>
+        <v/>
+      </c>
+      <c r="H28" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_FISCAL_Q", IQ_FQ - 2)</f>
+        <v/>
+      </c>
+      <c r="I28" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_FISCAL_Q", IQ_FQ - 1)</f>
+        <v/>
+      </c>
+      <c r="J28" s="97">
+        <f>_xll.ciqfunctions.udf.CIQ(Snapshot!C3, "IQ_FISCAL_Q", IQ_FQ)</f>
+        <v/>
+      </c>
+      <c r="K28" s="97" t="inlineStr">
+        <is>
+          <t>TR.FiscalQuarter</t>
         </is>
       </c>
     </row>

</xml_diff>